<commit_message>
Add extended INFOR Cap Table Template to repo
PR #27 bumped the captable-infor skill to v1.7.0 with new row references
for the extended template, but the template file itself was never
committed — the repo still had the old 141-row version. That caused the
skill to keep producing output against the old row map because the
plugin cache was pulling the stale template.

This commit replaces the template xlsx with the extended version
(190 rows; Section II: 57-81, III: 90-103, IV: 108-121, V: 126-142,
VI: 147-163, VII: 168-185) so SKILL.md v1.7.0 and the template agree.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/infor-workflows/templates/INFOR Cap Table Template.xlsx
+++ b/infor-workflows/templates/INFOR Cap Table Template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://inforfg1-my.sharepoint.com/personal/twilson_inforfg_com/Documents/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://inforfg1-my.sharepoint.com/personal/twilson_inforfg_com/Documents/Desktop/Claude Access Folder/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="151" documentId="13_ncr:1_{30C6EFFA-4D5C-4E44-9B68-CEAB259F3D95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{77F4C14A-FD65-4163-B92A-E6D3C1110A0F}"/>
+  <xr:revisionPtr revIDLastSave="210" documentId="13_ncr:1_{30C6EFFA-4D5C-4E44-9B68-CEAB259F3D95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{90EB48F8-F92B-4E4F-A9CF-26AEB629801A}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="__snloffice" sheetId="8" state="veryHidden" r:id="rId1"/>
@@ -50,7 +50,7 @@
     <definedName name="IQ_WEEK">50000</definedName>
     <definedName name="IQ_YTD">3000</definedName>
     <definedName name="IQ_YTDMONTH" hidden="1">130000</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'Cap with Links'!$A$1:$T$138</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Cap with Links'!$A$1:$T$187</definedName>
   </definedNames>
   <calcPr calcId="191029" iterate="1"/>
   <extLst>
@@ -286,7 +286,7 @@
     <t xml:space="preserve"> </t>
   </si>
   <si>
-    <t>允䅁䑁䅧䅁慁䅁䅁睔睂䡁䅑兡療䝁䄴督㙁䕁䄴兑㥁䑁䅁䅁汁䅁䅁䅅䅁䍁䅑睑䉂䕁䅑兖呂䕁䅑䅁䅁䅁䅁杈䅁䙁䅍䅕時䙁䅁杕䩂䕁䅍兒時䕁䅍䅔偂䙁䅍兒䅁䅁䅍䅁捁䅁䅁睔睂䡁䅑兡療䝁䄴督㙁䍁䅁杔䉂䑁䄰䅍䅁䅁䅑䅁䍁䅁䅁䅁剁䅁䅁䅏䅁䍁䅍兓佂䙁䅙兑䵂䕁䅫䅒杁䕁䅙兖佂䕁䅍䅖䩂䕁䄸杔杁䙁䅁兑卂䕁䅅兔䙂䙁䅑兒卂䅁䅁睄䅁䕁䅧䅁偂䡁䅁䅤灂䝁䄸杢穂䑁䅯兔桂䝁䅣児乂䝁䅫䅢獂䝁䅫睢畂䡁䅍䅌佂䕁䅅児佂䕁䅅䅌䑂䡁䅕杣祂䑁䄰兖呂䕁䅑䅁潁䅁䅁䅅䅁䕁䅙兕ぁ䑁䅉䅍祁䑁䅑䅁十䅁䅁杄䅁䕁䅍兗祁䑁䅁杍ㅁ䅁䅁睈䅁䅁䅧䅁䝂䙁䅅䅍䅁䅁䄰䅁佁䅁䅁睑婂䑁䅉䅍祁䑁䅙䅁楁䅁䅁䅅䅁䙁䅑睕奂䑁䅯兒䑂䕁䄴䅁煁䅁䅁杅䅁䕁䄴兗呂䕁䅕杏䩂䕁䅉兔䅁䉁䅍䅁佁䅁䅁睑婂䑁䅉䅍祁䑁䅣䅁桁䅁䅁䅉䅁䙁䅍䅕時䕁䅍睔乂䙁䅁兑佂䙁䅫睘佂䕁䅅兔䙂䅁䅁睂䅁䉁䅁䅁䝂䙁䅅免祁䑁䅁杍ㅁ䅁䅁䅅䅁䉁䅉䅁啂䙁䅍䅗㙁䕁䄸䅖䙂䙁䅧䅁牁䅁䅁䅅䅁䕁䅙兕祁䑁䅉䅍祁䑁䅕䅁橁䅁䅁杂䅁䕁䄴兑䅁䅁䅉䅁䥁䅁䅁杒婂䑁䅁䅁䭁䅁䅁䅈䅁䕁䅫兕時䕁䅅村呂䙁䄸䅕䙂䙁䅉兓偂䕁䅑䅁歁䅁䅁杌䅁䕁䅫兕時䕁䅍兖卂䙁䅉兒佂䕁䅍兗時䕁䅙兓佂䕁䅅杔䑂䕁䅫兑䵂䙁䅍䅁䱁䅁䅁杈䅁䙁䅍䅕時䕁䄴兖乂䙁䄸䅔偂䙁䅣睘卂䕁䅕睑䅁䉁䅯䅁流䅁䅁睕兂䙁䄸杔噂䕁䄰睘䥂䕁䅫睒䥂䕁䅕睕啂䙁䄸杕䙂䕁䅍䅁塁䅁䅁䅈䅁䕁䅫兕時䙁䅁兒卂䕁䅫睔䕂䙁䄸兒佂䕁䅑䅁䩁䅁䅁䅎䅁䕁䅫兕時䕁䅕睕啂䙁䄸杔䙂䙁䅧䅖時䕁䅕兑卂䕁䄴兓佂䕁䅣睕時䕁䅑兑啂䕁䅕䅁睁䅁䅁䅗䅁䕁䅫杢あ䝁䅕杣畂䝁䅅䅤灂䝁䄸杢桂䝁䅷䅉䍂䡁䅕督灂䝁䄴党穂䡁䅍䅉乂䝁䅅睙潂䝁䅫杢求䡁䅍䅉䑂䝁䄸杣睂䝁䄸杣桂䡁䅑兡療䝁䄴䅁湁䅁䅁杇䅁䕁䄴兑呂䕁䅑兑剂䕁䅍兔㙁䙁䅁村乂䅁䅁杂䅁䉁䄴䅁偂䡁䅁䅤灂䝁䄸杢穂䑁䅯䅉佂䕁䅅児佂䕁䅅䅁䙁䅁䅁䅌䅁䕁䅫兕時䕁䄴兒奂䙁䅑睘䙂䕁䅅杕佂䕁䅫杔䡂䙁䅍睘䕂䕁䅅䅖䙂䅁䅁兌䅁䑁䅁䅁偂䡁䅁䅤灂䝁䄸杢穂䑁䅯䅉佂䕁䅅児佂䕁䅅䅌䑂䙁䅕杕卂䑁䄰兖呂䕁䅑䅁摁䅁䅁䅍䅁䕁䄸䅣あ䝁䅫睢畂䡁䅍杏杁䕁䄴兑㥁䕁䄴兑獁䕁䅍兤祂䡁䅉児噂䙁䅍䅒䅁䉁䅑䅁奁䅁䅁睔睂䡁䅑兡療䝁䄴督㙁䕁䄴兑㥁䅁䅁杊䅁䍁䅧䅁橁䕁䅫杔坂䕁䅅䅔䩂䕁䅑䅉䑂䕁䄸兔兂䕁䅅杔婂䍁䅁兓䕂䅁䅁兎䅁䍁䅁䅁呂䙁䅁睘兂䙁䅉兓䑂䕁䅕睘啂䕁䅅杕䡂䕁䅕䅖䅁䉁䅷䅁捁䅁䅁睔睂䡁䅑兡療䝁䄴督㙁䕁䄴兑㥁䕁䄴兑䅁䉁䅙䅁䥁䅁䅁兖呂䕁䅑䅁䵁䅁䅁杌䅁䕁䄸䅣あ䝁䅫睢畂䡁䅍杏佂䕁䅅児佂䕁䅅䅌䑂䡁䅕杣祂䑁䄰兖呂䕁䅑䅁灁䅁䅁䅍䅁䙁䅁督㕂䝁䅕杢橂䝁䅕䅉䍂䝁䅫睢瑂䝁䅕䅚灂䝁䅍兙獂䍁䅁䅔あ䝁䅑杌䅁䅁䅧䅁杁䅁䅁睕兂䙁䄸杔噂䕁䄰睘䥂䕁䅫睒䥂䙁䄸杕䙂䕁䅍䅁奁䅁䅁䅎䅁䙁䅍䅕時䕁䅕兑卂䕁䄴兓佂䕁䅣睕時䕁䅅杔佂䕁䄸兖佂䕁䅍兒時䕁䅑兑啂䕁䅕䅁佁䅁䅁䅈䅁䙁䅍䅕時䕁䅕村䩂䙁䅑䅒䉂䙁䄸兒呂䙁䅑䅁杁䅁䅁杉䅁䙁䅍䅕時䕁䅷兑呂䙁䅑睕䉂䕁䅷兒兂䙁䅉兓䑂䕁䅕䅁䉁䅁䅁䅊䅁䙁䅍䅕時䕁䄴兖乂䙁䄸村卂䕁䄸睓䙂䙁䅉睘卂䕁䅕睑䅁䉁䅕䅁歁䅁䅁睕兂䙁䄸杔噂䕁䄰睘䵂䕁䄸睖䙂䙁䅍䅖時䙁䅉兒䑂䅁䅁睇䅁䍁䅙䅁呂䙁䅁睘佂䙁䅕兔時䕁䄴兒噂䙁䅑杕䉂䕁䅷睘卂䕁䅕睑䅁䉁䅫䅁坁䅁䅁睕兂䙁䄸杕䙂䙁䅙睘䙂䙁䅍䅖䅁䉁䄴䅁獁䅁䅁睔睂䝁䅕杢杁䙁䅑党㑂䡁䅑䅉䑂䝁䄸杣睂䝁䄸杣桂䡁䅑兡療䝁䄴䅁獁䅁䅁杆䅁䑁䅅免癁䑁䅅睍癁䑁䅉䅍祁䑁䅕䅁癁䅁䅁䅎䅁䕁䅫兕時䕁䅕兑卂䕁䄴兓佂䕁䅣睕時䕁䅅杔佂䕁䄸兖佂䕁䅍兒時䕁䅑兑啂䕁䅕䅁畁䅁䅁杄䅁䕁䅫兕時䙁䅉兒坂䅁䅁免䅁䅁䅧䅁䵂䙁䅑兔䅁䑁䅉䅁啁䅁䅁睕兂䙁䄸兒䍂䕁䅫䅖䕂䕁䅅䅁穁䅁䅁䅅䅁䍁䅑睑䉂䕁䅑睑䉂䕁䅑䅁ぁ䅁䅁杌䅁䕁䄸䅣あ䝁䅫睢畂䡁䅍杏佂䕁䅅児佂䕁䅅䅌䑂䡁䅕杣祂䑁䄰睑䉂䕁䅑䅁㉁䅁䅁䅓䅁䕁䄸䅣あ䝁䅫睢畂䡁䅍杏乂䝁䅅睚㥁䕁䄰兡獂䝁䅷兡療䝁䄴督獁䕁䄴兑㥁䕁䄴兑獁䕁䅍兤祂䡁䅉児䑂䕁䅅䅒䅁䑁䅣䅁䅁䅁䅁</t>
+    <t>允䅁䑁䅧䅁敁䅁䅁睕兂䙁䄸䅕卂䕁䅫睑䙂䙁䄸睑䵂䕁䄸睕䙂䅁䅁睁䅁䉁䅷䅁偂䡁䅁䅤灂䝁䄸杢穂䑁䅯䅉佂䕁䅅児睁䅁䅁䅂䅁䅁䅉䅁䅁䉁䅅䅁慁䅁䅁睔睂䡁䅑兡療䝁䄴督㙁䕁䄴兑㥁䑁䅁䅁汁䅁䅁䅅䅁䍁䅑睑䉂䕁䅑兖呂䕁䅑䅁䅁䅁䅁䅏䅁䍁䅍兓佂䙁䅙兑䵂䕁䅫䅒杁䕁䅙兖佂䕁䅍䅖䩂䕁䄸杔杁䙁䅁兑卂䕁䅅兔䙂䙁䅑兒卂䅁䅁睄䅁䅁䅧䅁䝂䙁䅅䅍䅁䅁䄰䅁佁䅁䅁睑婂䑁䅉䅍祁䑁䅕䅁晁䅁䅁䅓䅁䕁䄸䅣あ䝁䅫睢畂䡁䅍杏乂䝁䅅睚㥁䕁䄰兡獂䝁䅷兡療䝁䄴督獁䕁䄴兑㥁䕁䄴兑獁䕁䅍兤祂䡁䅉児噂䙁䅍䅒䅁䍁䅧䅁允䅁䅁杒剂䑁䅑杍睁䑁䅉䅎䅁䉁䅉䅁佁䅁䅁睑婂䑁䅉䅍祁䑁䅙䅁楁䅁䅁杄䅁䕁䅍兗祁䑁䅁杍㍁䅁䅁光䅁䉁䅉䅁佂䙁䅫睕䙂䑁䅯兓䍂䕁䄰䅁呁䅁䅁䅅䅁䙁䅑睕奂䑁䅯兒䑂䕁䄴䅁煁䅁䅁杅䅁䙁䅑睕奂䑁䅯睔啂䕁䅕䅗䅁䍁䅳䅁允䅁䅁杒剂䑁䅅杍睁䑁䅉兎䅁䉁䅁䅁杁䅁䅁睕兂䙁䄸睑偂䕁䄰䅕䉂䕁䄴兗時䕁䄴兑乂䕁䅕䅁䡁䅁䅁䅅䅁䕁䅙兕祁䑁䅉䅍祁䑁䅕䅁橁䅁䅁䅃䅁䕁䅙兗睁䅁䅁权䅁䅁䅙䅁佂䕁䅅䅁䍁䅁䅁䅈䅁䕁䅫兕時䕁䅅村呂䙁䄸䅕䙂䙁䅉兓偂䕁䅑䅁歁䅁䅁杌䅁䕁䅫兕時䕁䅍兖卂䙁䅉兒佂䕁䅍兗時䕁䅙兓佂䕁䅅杔䑂䕁䅫兑䵂䙁䅍䅁䱁䅁䅁䅎䅁䕁䅫兕時䕁䅕睕啂䙁䄸杔䙂䙁䅧䅖時䕁䅕兑卂䕁䄴兓佂䕁䅣睕時䕁䅑兑啂䕁䅕䅁睁䅁䅁䅈䅁䕁䅫兕時䙁䅁兒卂䕁䅫睔䕂䙁䄸兒佂䕁䅑䅁䩁䅁䅁杊䅁䙁䅍䅕時䕁䄴兖乂䙁䄸䅓䩂䕁䅣䅓䙂䙁䅍䅖時䙁䅉兒䑂䅁䅁睆䅁䉁䄴䅁呂䙁䅁睘佂䙁䅕兔時䕁䅷睔塂䙁䄸杕䙂䕁䅍䅁慁䅁䅁䅗䅁䕁䅫杢あ䝁䅕杣畂䝁䅅䅤灂䝁䄸杢桂䝁䅷䅉䍂䡁䅕督灂䝁䄴党穂䡁䅍䅉乂䝁䅅睙潂䝁䅫杢求䡁䅍䅉䑂䝁䄸杣睂䝁䄸杣桂䡁䅑兡療䝁䄴䅁湁䅁䅁杇䅁䕁䄴兑呂䕁䅑兑剂䕁䅍兔㙁䙁䅁村乂䅁䅁杂䅁䍁䅷䅁䩂䙁䅅睘佂䕁䅕䅗啂䙁䄸兒䉂䙁䅉杔䩂䕁䄴睒呂䙁䄸䅒䉂䙁䅑兒䅁䍁䄰䅁敁䅁䅁睔睂䡁䅑兡療䝁䄴督㙁䍁䅁杔䉂䑁䄰杔䉂䅁䅁兂䅁䑁䅁䅁偂䡁䅁䅤灂䝁䄸杢穂䑁䅯䅉佂䕁䅅児佂䕁䅅䅌䑂䙁䅕杕卂䑁䄰兖呂䕁䅑䅁摁䅁䅁䅍䅁䕁䄸䅣あ䝁䅫睢畂䡁䅍杏杁䕁䄴兑㥁䕁䄴兑獁䕁䅍兤祂䡁䅉児噂䙁䅍䅒䅁䉁䅑䅁潁䅁䅁睉䩂䕁䄴杖䉂䕁䅷兓䕂䍁䅁睑偂䕁䄰䅕䉂䕁䄴兗杁䕁䅫䅒䅁䑁䅕䅁奁䅁䅁睔睂䡁䅑兡療䝁䄴督㙁䕁䄴兑㥁䅁䅁杊䅁䉁䅷䅁偂䡁䅁䅤灂䝁䄸杢穂䑁䅯杔䉂䑁䄰杔䉂䅁䅁杆䅁䍁䅁䅁呂䙁䅁睘兂䙁䅉兓䑂䕁䅕睘啂䕁䅅杕䡂䕁䅕䅖䅁䉁䅷䅁畁䅁䅁睔睂䡁䅑兡療䝁䄴督㙁䕁䄴兑㥁䕁䄴兑獁䕁䅍兤祂䡁䅉児噂䙁䅍䅒䅁䍁䅫䅁䥁䅁䅁兖呂䕁䅑䅁䵁䅁䅁䅍䅁䙁䅁督㕂䝁䅕杢橂䝁䅕䅉䍂䝁䅫睢瑂䝁䅕䅚灂䝁䅍兙獂䍁䅁䅔あ䝁䅑杌䅁䅁䅧䅁ぁ䅁䅁睕兂䙁䄸兒䉂䙁䅉杔䩂䕁䄴睒呂䙁䄸兑佂䕁䄴睔噂䕁䄴睑䙂䙁䄸䅒䉂䙁䅑兒䅁䅁䄴䅁杁䅁䅁睕兂䙁䄸杔噂䕁䄰睘䥂䕁䅫睒䥂䙁䄸杕䙂䕁䅍䅁奁䅁䅁䅈䅁䙁䅍䅕時䕁䅕村䩂䙁䅑䅒䉂䙁䄸兒呂䙁䅑䅁杁䅁䅁杉䅁䙁䅍䅕時䕁䅷兑呂䙁䅑睕䉂䕁䅷兒兂䙁䅉兓䑂䕁䅕䅁䉁䅁䅁䅊䅁䙁䅍䅕時䕁䄴兖乂䙁䄸村卂䕁䄸睓䙂䙁䅉睘卂䕁䅕睑䅁䉁䅕䅁歁䅁䅁睕兂䙁䄸杔噂䕁䄰睘䵂䕁䄸睖䙂䙁䅍䅖時䙁䅉兒䑂䅁䅁睇䅁䍁䅙䅁呂䙁䅁睘佂䙁䅕兔時䕁䄴兒噂䙁䅑杕䉂䕁䅷睘卂䕁䅕睑䅁䉁䅫䅁坁䅁䅁睕兂䙁䄸杕䙂䙁䅙睘䙂䙁䅍䅖䅁䉁䄴䅁坁䅁䅁免硁䍁䄸免穁䍁䄸杍睁䑁䅉兎䅁䍁䄸䅁獁䅁䅁睔睂䝁䅕杢杁䙁䅑党㑂䡁䅑䅉䑂䝁䄸杣睂䝁䄸杣桂䡁䅑兡療䝁䄴䅁獁䅁䅁䅎䅁䕁䅫兕時䕁䅕兑卂䕁䄴兓佂䕁䅣睕時䕁䅅杔佂䕁䄸兖佂䕁䅍兒時䕁䅑兑啂䕁䅕䅁畁䅁䅁杄䅁䕁䅫兕時䙁䅉兒坂䅁䅁免䅁䅁䅧䅁䵂䙁䅑兔䅁䑁䅉䅁啁䅁䅁睕兂䙁䄸兒䍂䕁䅫䅖䕂䕁䅅䅁穁䅁䅁䅅䅁䍁䅑睑䉂䕁䅑睑䉂䕁䅑䅁ぁ䅁䅁杌䅁䕁䄸䅣あ䝁䅫睢畂䡁䅍杏佂䕁䅅児佂䕁䅅䅌䑂䡁䅕杣祂䑁䄰睑䉂䕁䅑䅁㉁䅁䅁䅓䅁䕁䄸䅣あ䝁䅫睢畂䡁䅍杏乂䝁䅅睚㥁䕁䄰兡獂䝁䅷兡療䝁䄴督獁䕁䄴兑㥁䕁䄴兑獁䕁䅍兤祂䡁䅉児䑂䕁䅅䅒䅁䑁䅣䅁䅁䅁䅁</t>
   </si>
 </sst>
 </file>
@@ -1414,7 +1414,7 @@
 
 <file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
 <wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
-  <wetp:taskpane dockstate="right" visibility="0" width="350" row="7">
+  <wetp:taskpane dockstate="right" visibility="0" width="350" row="3">
     <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </wetp:taskpane>
 </wetp:taskpanes>
@@ -1428,6 +1428,7 @@
   </we:alternateReferences>
   <we:properties>
     <we:property name="Office.AutoShowTaskpaneWithDocument" value="true"/>
+    <we:property name="claude.fileId" value="&quot;01b1f51b-2e76-480b-a0db-905fabf74c22&quot;"/>
   </we:properties>
   <we:bindings/>
   <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
@@ -1452,7 +1453,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Sheet2"/>
-  <dimension ref="A1:Q141"/>
+  <dimension ref="A1:Q190"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="2.7109375" style="4" customWidth="1"/>
@@ -1535,7 +1536,7 @@
       <c r="E6" s="87"/>
       <c r="F6" s="93">
         <f ca="1">TODAY()-1</f>
-        <v>46098</v>
+        <v>46133</v>
       </c>
       <c r="H6" s="66"/>
     </row>
@@ -1637,7 +1638,7 @@
     <row r="16" spans="1:10" s="4" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="111" t="str">
         <f ca="1">CONCATENATE("Share Price (",TEXT(F6,"dd-mmm-yy"),")")</f>
-        <v>Share Price (17-Mar-26)</v>
+        <v>Share Price (21-Apr-26)</v>
       </c>
       <c r="F16" s="125" t="str" cm="1">
         <f t="array" aca="1" ref="F16" ca="1">_xll.SNL.Clients.Office.Excel.Functions.SPG($F$3,"SP_LASTSALEPRICE",$F$6,"Options:NA=NA,Curr="&amp;$F$5)</f>
@@ -1650,7 +1651,7 @@
         <v>4</v>
       </c>
       <c r="F17" s="124">
-        <f>F137</f>
+        <f>F186</f>
         <v>0</v>
       </c>
     </row>
@@ -1681,7 +1682,7 @@
         <v>Net ITM Dilutive Securities</v>
       </c>
       <c r="F19" s="124" t="e">
-        <f ca="1">IF(F10="Treasury Stock",F77,F75)</f>
+        <f ca="1">IF(F10="Treasury Stock",F86,F84)</f>
         <v>#VALUE!</v>
       </c>
     </row>
@@ -1690,7 +1691,7 @@
         <v>6</v>
       </c>
       <c r="F20" s="124">
-        <f ca="1">F87</f>
+        <f ca="1">F104</f>
         <v>0</v>
       </c>
     </row>
@@ -1755,7 +1756,7 @@
         <v>27</v>
       </c>
       <c r="F24" s="109" t="e">
-        <f ca="1">F99*F7</f>
+        <f ca="1">F122*F7</f>
         <v>#VALUE!</v>
       </c>
       <c r="I24" s="3"/>
@@ -1773,7 +1774,7 @@
         <v>42</v>
       </c>
       <c r="F25" s="109" t="e">
-        <f ca="1">IF($F$11="ON",$F$111,0)*F7</f>
+        <f ca="1">IF($F$11="ON",$F$143,0)*F7</f>
         <v>#VALUE!</v>
       </c>
       <c r="I25" s="3"/>
@@ -1791,7 +1792,7 @@
         <v>7</v>
       </c>
       <c r="F26" s="109" t="e">
-        <f ca="1">-F123*F7</f>
+        <f ca="1">-F164*F7</f>
         <v>#VALUE!</v>
       </c>
       <c r="I26" s="3"/>
@@ -1809,7 +1810,7 @@
         <v>43</v>
       </c>
       <c r="F27" s="109" t="e">
-        <f ca="1">IF(F10="Treasury Stock",0,-F73)*F7</f>
+        <f ca="1">IF(F10="Treasury Stock",0,-F82)*F7</f>
         <v>#VALUE!</v>
       </c>
       <c r="I27" s="3"/>
@@ -2144,15 +2145,15 @@
       </c>
       <c r="H48" s="66"/>
     </row>
-    <row r="49" spans="2:8" s="4" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="2:17" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B49" s="12"/>
       <c r="C49" s="10"/>
       <c r="D49" s="61"/>
       <c r="E49" s="61"/>
       <c r="F49" s="61"/>
-      <c r="H49" s="66"/>
-    </row>
-    <row r="50" spans="2:8" s="4" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="Q49" s="4"/>
+    </row>
+    <row r="50" spans="2:17" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B50" s="79" t="s">
         <v>52</v>
       </c>
@@ -2160,9 +2161,9 @@
       <c r="D50" s="80"/>
       <c r="E50" s="80"/>
       <c r="F50" s="80"/>
-      <c r="H50" s="66"/>
-    </row>
-    <row r="51" spans="2:8" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="Q50" s="4"/>
+    </row>
+    <row r="51" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B51" s="81" t="s">
         <v>9</v>
       </c>
@@ -2174,34 +2175,34 @@
       <c r="F51" s="84" t="s">
         <v>10</v>
       </c>
-      <c r="H51" s="66"/>
-    </row>
-    <row r="52" spans="2:8" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="Q51" s="4"/>
+    </row>
+    <row r="52" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B52" s="77" t="s">
         <v>26</v>
       </c>
       <c r="D52" s="13"/>
       <c r="E52" s="31"/>
       <c r="F52" s="48"/>
-      <c r="H52" s="66"/>
-    </row>
-    <row r="53" spans="2:8" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="Q52" s="4"/>
+    </row>
+    <row r="53" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B53" s="77" t="s">
         <v>25</v>
       </c>
       <c r="D53" s="13"/>
       <c r="E53" s="31"/>
       <c r="F53" s="48"/>
-      <c r="H53" s="66"/>
-    </row>
-    <row r="54" spans="2:8" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="Q53" s="4"/>
+    </row>
+    <row r="54" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B54" s="12"/>
       <c r="D54" s="13"/>
       <c r="E54" s="13"/>
       <c r="F54" s="23"/>
-      <c r="H54" s="66"/>
-    </row>
-    <row r="55" spans="2:8" s="4" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="Q54" s="4"/>
+    </row>
+    <row r="55" spans="2:17" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B55" s="79" t="s">
         <v>37</v>
       </c>
@@ -2209,9 +2210,9 @@
       <c r="D55" s="80"/>
       <c r="E55" s="80"/>
       <c r="F55" s="80"/>
-      <c r="H55" s="66"/>
-    </row>
-    <row r="56" spans="2:8" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="Q55" s="4"/>
+    </row>
+    <row r="56" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B56" s="81" t="s">
         <v>9</v>
       </c>
@@ -2227,9 +2228,9 @@
       <c r="F56" s="84" t="s">
         <v>13</v>
       </c>
-      <c r="H56" s="66"/>
-    </row>
-    <row r="57" spans="2:8" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="Q56" s="4"/>
+    </row>
+    <row r="57" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B57" s="24"/>
       <c r="C57" s="25"/>
       <c r="D57" s="26"/>
@@ -2241,23 +2242,24 @@
         <f ca="1">E57*D57</f>
         <v>0</v>
       </c>
-      <c r="H57" s="66"/>
-    </row>
-    <row r="58" spans="2:8" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="Q57" s="4"/>
+    </row>
+    <row r="58" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B58" s="24"/>
       <c r="C58" s="25"/>
       <c r="D58" s="26"/>
       <c r="E58" s="45">
-        <f t="shared" ref="E58:E72" ca="1" si="3">IF(D58&lt;F$16,C58,0)</f>
+        <f t="shared" ref="E58:E81" ca="1" si="3">IF(D58&lt;F$16,C58,0)</f>
         <v>0</v>
       </c>
       <c r="F58" s="44">
-        <f t="shared" ref="F58:F72" ca="1" si="4">E58*D58</f>
+        <f t="shared" ref="F58:F81" ca="1" si="4">E58*D58</f>
         <v>0</v>
       </c>
       <c r="H58" s="71"/>
-    </row>
-    <row r="59" spans="2:8" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="Q58" s="4"/>
+    </row>
+    <row r="59" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B59" s="24"/>
       <c r="C59" s="25"/>
       <c r="D59" s="26"/>
@@ -2270,8 +2272,9 @@
         <v>0</v>
       </c>
       <c r="H59" s="71"/>
-    </row>
-    <row r="60" spans="2:8" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="Q59" s="4"/>
+    </row>
+    <row r="60" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B60" s="24"/>
       <c r="C60" s="25"/>
       <c r="D60" s="26"/>
@@ -2283,9 +2286,9 @@
         <f t="shared" ca="1" si="4"/>
         <v>0</v>
       </c>
-      <c r="H60" s="66"/>
-    </row>
-    <row r="61" spans="2:8" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="Q60" s="4"/>
+    </row>
+    <row r="61" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B61" s="24"/>
       <c r="C61" s="25"/>
       <c r="D61" s="26"/>
@@ -2297,9 +2300,9 @@
         <f t="shared" ca="1" si="4"/>
         <v>0</v>
       </c>
-      <c r="H61" s="66"/>
-    </row>
-    <row r="62" spans="2:8" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="Q61" s="4"/>
+    </row>
+    <row r="62" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B62" s="24"/>
       <c r="C62" s="25"/>
       <c r="D62" s="26"/>
@@ -2311,9 +2314,9 @@
         <f t="shared" ca="1" si="4"/>
         <v>0</v>
       </c>
-      <c r="H62" s="66"/>
-    </row>
-    <row r="63" spans="2:8" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="Q62" s="4"/>
+    </row>
+    <row r="63" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B63" s="24"/>
       <c r="C63" s="25"/>
       <c r="D63" s="26"/>
@@ -2325,9 +2328,9 @@
         <f t="shared" ca="1" si="4"/>
         <v>0</v>
       </c>
-      <c r="H63" s="66"/>
-    </row>
-    <row r="64" spans="2:8" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="Q63" s="4"/>
+    </row>
+    <row r="64" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B64" s="24"/>
       <c r="C64" s="25"/>
       <c r="D64" s="26"/>
@@ -2339,59 +2342,63 @@
         <f t="shared" ca="1" si="4"/>
         <v>0</v>
       </c>
-      <c r="H64" s="66"/>
+      <c r="Q64" s="4"/>
     </row>
     <row r="65" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B65" s="24"/>
       <c r="C65" s="25"/>
       <c r="D65" s="26"/>
       <c r="E65" s="45">
-        <f t="shared" ca="1" si="3"/>
+        <f t="shared" ref="E65:E74" ca="1" si="5">IF(D65&lt;F$16,C65,0)</f>
         <v>0</v>
       </c>
       <c r="F65" s="44">
-        <f t="shared" ca="1" si="4"/>
-        <v>0</v>
-      </c>
+        <f t="shared" ref="F65:F74" ca="1" si="6">E65*D65</f>
+        <v>0</v>
+      </c>
+      <c r="Q65" s="4"/>
     </row>
     <row r="66" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B66" s="24"/>
       <c r="C66" s="25"/>
       <c r="D66" s="26"/>
       <c r="E66" s="45">
-        <f t="shared" ca="1" si="3"/>
+        <f t="shared" ca="1" si="5"/>
         <v>0</v>
       </c>
       <c r="F66" s="44">
-        <f t="shared" ca="1" si="4"/>
-        <v>0</v>
-      </c>
+        <f t="shared" ca="1" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="Q66" s="4"/>
     </row>
     <row r="67" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B67" s="24"/>
       <c r="C67" s="25"/>
       <c r="D67" s="26"/>
       <c r="E67" s="45">
-        <f ca="1">IF(D67&lt;F$16,C67,0)</f>
+        <f t="shared" ca="1" si="5"/>
         <v>0</v>
       </c>
       <c r="F67" s="44">
-        <f t="shared" ca="1" si="4"/>
-        <v>0</v>
-      </c>
+        <f t="shared" ca="1" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="Q67" s="4"/>
     </row>
     <row r="68" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B68" s="24"/>
       <c r="C68" s="25"/>
       <c r="D68" s="26"/>
       <c r="E68" s="45">
-        <f t="shared" ref="E68:E71" ca="1" si="5">IF(D68&lt;F$16,C68,0)</f>
+        <f t="shared" ca="1" si="5"/>
         <v>0</v>
       </c>
       <c r="F68" s="44">
-        <f t="shared" ca="1" si="4"/>
-        <v>0</v>
-      </c>
+        <f t="shared" ca="1" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="Q68" s="4"/>
     </row>
     <row r="69" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B69" s="24"/>
@@ -2402,9 +2409,10 @@
         <v>0</v>
       </c>
       <c r="F69" s="44">
-        <f t="shared" ca="1" si="4"/>
-        <v>0</v>
-      </c>
+        <f t="shared" ca="1" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="Q69" s="4"/>
     </row>
     <row r="70" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B70" s="24"/>
@@ -2415,9 +2423,10 @@
         <v>0</v>
       </c>
       <c r="F70" s="44">
-        <f t="shared" ca="1" si="4"/>
-        <v>0</v>
-      </c>
+        <f t="shared" ca="1" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="Q70" s="4"/>
     </row>
     <row r="71" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B71" s="24"/>
@@ -2428,406 +2437,446 @@
         <v>0</v>
       </c>
       <c r="F71" s="44">
-        <f t="shared" ca="1" si="4"/>
-        <v>0</v>
-      </c>
+        <f t="shared" ca="1" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="Q71" s="4"/>
     </row>
     <row r="72" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B72" s="24"/>
       <c r="C72" s="25"/>
       <c r="D72" s="26"/>
       <c r="E72" s="45">
+        <f t="shared" ca="1" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="F72" s="44">
+        <f t="shared" ca="1" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="Q72" s="4"/>
+    </row>
+    <row r="73" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B73" s="24"/>
+      <c r="C73" s="25"/>
+      <c r="D73" s="26"/>
+      <c r="E73" s="45">
+        <f t="shared" ca="1" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="F73" s="44">
+        <f t="shared" ca="1" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="Q73" s="4"/>
+    </row>
+    <row r="74" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B74" s="24"/>
+      <c r="C74" s="25"/>
+      <c r="D74" s="26"/>
+      <c r="E74" s="45">
+        <f t="shared" ca="1" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="F74" s="44">
+        <f t="shared" ca="1" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="Q74" s="4"/>
+    </row>
+    <row r="75" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B75" s="24"/>
+      <c r="C75" s="25"/>
+      <c r="D75" s="26"/>
+      <c r="E75" s="45">
         <f t="shared" ca="1" si="3"/>
         <v>0</v>
       </c>
-      <c r="F72" s="44">
+      <c r="F75" s="44">
         <f t="shared" ca="1" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="2:17" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B73" s="27" t="s">
-        <v>14</v>
-      </c>
-      <c r="C73" s="27"/>
-      <c r="D73" s="27"/>
-      <c r="E73" s="55">
-        <f ca="1">SUM(E57:E72)</f>
-        <v>0</v>
-      </c>
-      <c r="F73" s="47">
-        <f ca="1">SUM(F57:F72)</f>
-        <v>0</v>
-      </c>
-      <c r="H73" s="70"/>
-      <c r="Q73" s="28"/>
-    </row>
-    <row r="75" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B75" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="F75" s="45">
-        <f ca="1">E73</f>
-        <v>0</v>
-      </c>
-    </row>
     <row r="76" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B76" s="17" t="s">
-        <v>16</v>
-      </c>
-      <c r="C76" s="17"/>
-      <c r="D76" s="17"/>
-      <c r="E76" s="17"/>
-      <c r="F76" s="52" t="e">
-        <f ca="1">-F73/F16</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="77" spans="2:17" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B77" s="27" t="s">
-        <v>17</v>
-      </c>
-      <c r="C77" s="27"/>
-      <c r="D77" s="27"/>
-      <c r="E77" s="27"/>
-      <c r="F77" s="55" t="e">
-        <f ca="1">SUM(F75:F76)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="H77" s="70"/>
-      <c r="Q77" s="28"/>
-    </row>
-    <row r="79" spans="2:17" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B79" s="79" t="s">
-        <v>47</v>
-      </c>
-      <c r="C79" s="80"/>
-      <c r="D79" s="80"/>
-      <c r="E79" s="80"/>
-      <c r="F79" s="80"/>
+      <c r="B76" s="24"/>
+      <c r="C76" s="25"/>
+      <c r="D76" s="26"/>
+      <c r="E76" s="45">
+        <f ca="1">IF(D76&lt;F$16,C76,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F76" s="44">
+        <f t="shared" ca="1" si="4"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B77" s="24"/>
+      <c r="C77" s="25"/>
+      <c r="D77" s="26"/>
+      <c r="E77" s="45">
+        <f t="shared" ref="E77:E80" ca="1" si="7">IF(D77&lt;F$16,C77,0)</f>
+        <v>0</v>
+      </c>
+      <c r="F77" s="44">
+        <f t="shared" ca="1" si="4"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B78" s="24"/>
+      <c r="C78" s="25"/>
+      <c r="D78" s="26"/>
+      <c r="E78" s="45">
+        <f t="shared" ca="1" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="F78" s="44">
+        <f t="shared" ca="1" si="4"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B79" s="24"/>
+      <c r="C79" s="25"/>
+      <c r="D79" s="26"/>
+      <c r="E79" s="45">
+        <f t="shared" ca="1" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="F79" s="44">
+        <f t="shared" ca="1" si="4"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="80" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B80" s="81" t="s">
-        <v>9</v>
-      </c>
-      <c r="C80" s="83" t="s">
-        <v>10</v>
-      </c>
-      <c r="D80" s="83" t="s">
-        <v>53</v>
-      </c>
-      <c r="E80" s="83" t="s">
-        <v>11</v>
-      </c>
-      <c r="F80" s="84" t="s">
-        <v>12</v>
+      <c r="B80" s="24"/>
+      <c r="C80" s="25"/>
+      <c r="D80" s="26"/>
+      <c r="E80" s="45">
+        <f t="shared" ca="1" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="F80" s="44">
+        <f t="shared" ca="1" si="4"/>
+        <v>0</v>
       </c>
     </row>
     <row r="81" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B81" s="24"/>
-      <c r="C81" s="48"/>
-      <c r="D81" s="85"/>
-      <c r="E81" s="53"/>
-      <c r="F81" s="45">
-        <f t="shared" ref="F81:F86" ca="1" si="6">IF(E81&lt;F$16,(C81/1000)*D81,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="82" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B82" s="24"/>
-      <c r="C82" s="48"/>
-      <c r="D82" s="54"/>
-      <c r="E82" s="53"/>
-      <c r="F82" s="45">
-        <f ca="1">IF(E82&lt;F$16,(C82/1000)*D82,0)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="83" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B83" s="24"/>
-      <c r="C83" s="48"/>
-      <c r="D83" s="54"/>
-      <c r="E83" s="53"/>
-      <c r="F83" s="45">
-        <f ca="1">IF(E83&lt;F$16,(C83/1000)*D83,0)</f>
-        <v>0</v>
-      </c>
+      <c r="C81" s="25"/>
+      <c r="D81" s="26"/>
+      <c r="E81" s="45">
+        <f t="shared" ca="1" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="F81" s="44">
+        <f t="shared" ca="1" si="4"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82" spans="2:17" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B82" s="27" t="s">
+        <v>14</v>
+      </c>
+      <c r="C82" s="27"/>
+      <c r="D82" s="27"/>
+      <c r="E82" s="55">
+        <f ca="1">SUM(E57:E81)</f>
+        <v>0</v>
+      </c>
+      <c r="F82" s="47">
+        <f ca="1">SUM(F57:F81)</f>
+        <v>0</v>
+      </c>
+      <c r="H82" s="70"/>
+      <c r="Q82" s="28"/>
     </row>
     <row r="84" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B84" s="24"/>
-      <c r="C84" s="48"/>
-      <c r="D84" s="54"/>
-      <c r="E84" s="53"/>
+      <c r="B84" s="4" t="s">
+        <v>15</v>
+      </c>
       <c r="F84" s="45">
-        <f t="shared" ca="1" si="6"/>
+        <f ca="1">E82</f>
         <v>0</v>
       </c>
     </row>
     <row r="85" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B85" s="24"/>
-      <c r="C85" s="48"/>
-      <c r="D85" s="54"/>
-      <c r="E85" s="53"/>
-      <c r="F85" s="45">
-        <f t="shared" ca="1" si="6"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="86" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B86" s="24"/>
-      <c r="C86" s="48"/>
-      <c r="D86" s="54"/>
-      <c r="E86" s="53"/>
-      <c r="F86" s="45">
-        <f t="shared" ca="1" si="6"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="87" spans="2:17" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B87" s="27" t="s">
-        <v>18</v>
-      </c>
-      <c r="C87" s="27"/>
-      <c r="D87" s="27"/>
-      <c r="E87" s="27"/>
-      <c r="F87" s="55">
-        <f ca="1">SUM(F81:F86)</f>
-        <v>0</v>
-      </c>
-      <c r="H87" s="70"/>
-      <c r="Q87" s="28"/>
-    </row>
-    <row r="89" spans="2:17" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B89" s="79" t="s">
-        <v>19</v>
-      </c>
-      <c r="C89" s="80"/>
-      <c r="D89" s="80"/>
-      <c r="E89" s="80"/>
-      <c r="F89" s="80"/>
+      <c r="B85" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="C85" s="17"/>
+      <c r="D85" s="17"/>
+      <c r="E85" s="17"/>
+      <c r="F85" s="52" t="e">
+        <f ca="1">-F82/F16</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="86" spans="2:17" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B86" s="27" t="s">
+        <v>17</v>
+      </c>
+      <c r="C86" s="27"/>
+      <c r="D86" s="27"/>
+      <c r="E86" s="27"/>
+      <c r="F86" s="55" t="e">
+        <f ca="1">SUM(F84:F85)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="H86" s="70"/>
+      <c r="Q86" s="28"/>
+    </row>
+    <row r="88" spans="2:17" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B88" s="79" t="s">
+        <v>47</v>
+      </c>
+      <c r="C88" s="80"/>
+      <c r="D88" s="80"/>
+      <c r="E88" s="80"/>
+      <c r="F88" s="80"/>
+    </row>
+    <row r="89" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B89" s="81" t="s">
+        <v>9</v>
+      </c>
+      <c r="C89" s="83" t="s">
+        <v>10</v>
+      </c>
+      <c r="D89" s="83" t="s">
+        <v>53</v>
+      </c>
+      <c r="E89" s="83" t="s">
+        <v>11</v>
+      </c>
+      <c r="F89" s="84" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="90" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B90" s="81" t="s">
-        <v>9</v>
-      </c>
-      <c r="C90" s="82"/>
-      <c r="D90" s="82"/>
-      <c r="E90" s="83" t="s">
-        <v>0</v>
-      </c>
-      <c r="F90" s="84" t="s">
-        <v>10</v>
+      <c r="B90" s="24"/>
+      <c r="C90" s="48"/>
+      <c r="D90" s="85"/>
+      <c r="E90" s="53"/>
+      <c r="F90" s="45">
+        <f t="shared" ref="F90:F103" ca="1" si="8">IF(E90&lt;F$16,(C90/1000)*D90,0)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="91" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B91" s="24"/>
-      <c r="C91" s="29"/>
-      <c r="D91" s="30"/>
-      <c r="E91" s="31"/>
-      <c r="F91" s="48"/>
+      <c r="C91" s="48"/>
+      <c r="D91" s="54"/>
+      <c r="E91" s="53"/>
+      <c r="F91" s="45">
+        <f ca="1">IF(E91&lt;F$16,(C91/1000)*D91,0)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="92" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B92" s="24"/>
-      <c r="C92" s="29"/>
-      <c r="D92" s="30"/>
-      <c r="E92" s="31"/>
-      <c r="F92" s="48"/>
+      <c r="C92" s="48"/>
+      <c r="D92" s="54"/>
+      <c r="E92" s="53"/>
+      <c r="F92" s="45">
+        <f t="shared" ref="F92:F99" ca="1" si="9">IF(E92&lt;F$16,(C92/1000)*D92,0)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="93" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B93" s="75"/>
-      <c r="C93" s="29"/>
-      <c r="D93" s="30"/>
-      <c r="E93" s="31"/>
-      <c r="F93" s="48"/>
+      <c r="B93" s="24"/>
+      <c r="C93" s="48"/>
+      <c r="D93" s="54"/>
+      <c r="E93" s="53"/>
+      <c r="F93" s="45">
+        <f t="shared" ca="1" si="9"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="94" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B94" s="24"/>
-      <c r="C94" s="29"/>
-      <c r="D94" s="30"/>
-      <c r="E94" s="31"/>
-      <c r="F94" s="48"/>
+      <c r="C94" s="48"/>
+      <c r="D94" s="54"/>
+      <c r="E94" s="53"/>
+      <c r="F94" s="45">
+        <f t="shared" ca="1" si="9"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="95" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B95" s="24"/>
-      <c r="C95" s="29"/>
-      <c r="D95" s="30"/>
-      <c r="E95" s="31"/>
-      <c r="F95" s="48"/>
-      <c r="H95" s="4"/>
+      <c r="C95" s="48"/>
+      <c r="D95" s="54"/>
+      <c r="E95" s="53"/>
+      <c r="F95" s="45">
+        <f t="shared" ca="1" si="9"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="96" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B96" s="24"/>
-      <c r="C96" s="29"/>
-      <c r="D96" s="30"/>
-      <c r="E96" s="31"/>
-      <c r="F96" s="48"/>
+      <c r="C96" s="48"/>
+      <c r="D96" s="54"/>
+      <c r="E96" s="53"/>
+      <c r="F96" s="45">
+        <f t="shared" ca="1" si="9"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="97" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B97" s="24"/>
-      <c r="C97" s="29"/>
-      <c r="D97" s="30"/>
-      <c r="E97" s="31"/>
-      <c r="F97" s="48"/>
+      <c r="C97" s="48"/>
+      <c r="D97" s="54"/>
+      <c r="E97" s="53"/>
+      <c r="F97" s="45">
+        <f t="shared" ca="1" si="9"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="98" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B98" s="24"/>
-      <c r="C98" s="29"/>
-      <c r="D98" s="30"/>
-      <c r="E98" s="32"/>
-      <c r="F98" s="48"/>
-    </row>
-    <row r="99" spans="2:17" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B99" s="74" t="s">
-        <v>20</v>
-      </c>
-      <c r="C99" s="27"/>
-      <c r="D99" s="27"/>
-      <c r="E99" s="27"/>
-      <c r="F99" s="47">
-        <f>SUM(F91:F98)</f>
-        <v>0</v>
-      </c>
-      <c r="H99" s="70"/>
-      <c r="Q99" s="28"/>
-    </row>
-    <row r="100" spans="2:17" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="F100" s="64"/>
-      <c r="H100" s="70"/>
-      <c r="Q100" s="28"/>
-    </row>
-    <row r="101" spans="2:17" s="10" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B101" s="79" t="s">
-        <v>39</v>
-      </c>
-      <c r="C101" s="80"/>
-      <c r="D101" s="80"/>
-      <c r="E101" s="80"/>
-      <c r="F101" s="80"/>
-      <c r="H101" s="70"/>
-      <c r="Q101" s="28"/>
-    </row>
-    <row r="102" spans="2:17" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B102" s="81" t="s">
+      <c r="C98" s="48"/>
+      <c r="D98" s="54"/>
+      <c r="E98" s="53"/>
+      <c r="F98" s="45">
+        <f t="shared" ca="1" si="9"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="99" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B99" s="24"/>
+      <c r="C99" s="48"/>
+      <c r="D99" s="54"/>
+      <c r="E99" s="53"/>
+      <c r="F99" s="45">
+        <f t="shared" ca="1" si="9"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="100" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B100" s="24"/>
+      <c r="C100" s="48"/>
+      <c r="D100" s="54"/>
+      <c r="E100" s="53"/>
+      <c r="F100" s="45">
+        <f ca="1">IF(E100&lt;F$16,(C100/1000)*D100,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="101" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B101" s="24"/>
+      <c r="C101" s="48"/>
+      <c r="D101" s="54"/>
+      <c r="E101" s="53"/>
+      <c r="F101" s="45">
+        <f t="shared" ca="1" si="8"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="102" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B102" s="24"/>
+      <c r="C102" s="48"/>
+      <c r="D102" s="54"/>
+      <c r="E102" s="53"/>
+      <c r="F102" s="45">
+        <f t="shared" ca="1" si="8"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="103" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B103" s="24"/>
+      <c r="C103" s="48"/>
+      <c r="D103" s="54"/>
+      <c r="E103" s="53"/>
+      <c r="F103" s="45">
+        <f t="shared" ca="1" si="8"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="104" spans="2:17" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B104" s="27" t="s">
+        <v>18</v>
+      </c>
+      <c r="C104" s="27"/>
+      <c r="D104" s="27"/>
+      <c r="E104" s="27"/>
+      <c r="F104" s="55">
+        <f ca="1">SUM(F90:F103)</f>
+        <v>0</v>
+      </c>
+      <c r="H104" s="70"/>
+      <c r="Q104" s="28"/>
+    </row>
+    <row r="106" spans="2:17" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B106" s="79" t="s">
+        <v>19</v>
+      </c>
+      <c r="C106" s="80"/>
+      <c r="D106" s="80"/>
+      <c r="E106" s="80"/>
+      <c r="F106" s="80"/>
+    </row>
+    <row r="107" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B107" s="81" t="s">
         <v>9</v>
       </c>
-      <c r="C102" s="82"/>
-      <c r="D102" s="82"/>
-      <c r="E102" s="83" t="s">
-        <v>0</v>
-      </c>
-      <c r="F102" s="83" t="s">
+      <c r="C107" s="82"/>
+      <c r="D107" s="82"/>
+      <c r="E107" s="83" t="s">
+        <v>0</v>
+      </c>
+      <c r="F107" s="84" t="s">
         <v>10</v>
       </c>
-      <c r="H102" s="70"/>
-      <c r="Q102" s="28"/>
-    </row>
-    <row r="103" spans="2:17" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B103" s="24"/>
-      <c r="C103" s="29"/>
-      <c r="D103" s="30"/>
-      <c r="E103" s="31"/>
-      <c r="F103" s="48"/>
-      <c r="H103" s="66"/>
-      <c r="Q103" s="28"/>
-    </row>
-    <row r="104" spans="2:17" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B104" s="24"/>
-      <c r="C104" s="29"/>
-      <c r="D104" s="30"/>
-      <c r="E104" s="31"/>
-      <c r="F104" s="48"/>
-      <c r="H104" s="66"/>
-      <c r="Q104" s="28"/>
-    </row>
-    <row r="105" spans="2:17" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B105" s="24"/>
-      <c r="C105" s="29"/>
-      <c r="D105" s="30"/>
-      <c r="E105" s="31"/>
-      <c r="F105" s="48"/>
-      <c r="H105" s="66"/>
-      <c r="Q105" s="28"/>
-    </row>
-    <row r="106" spans="2:17" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B106" s="24"/>
-      <c r="C106" s="29"/>
-      <c r="D106" s="30"/>
-      <c r="E106" s="31"/>
-      <c r="F106" s="48"/>
-      <c r="H106" s="70"/>
-      <c r="Q106" s="28"/>
-    </row>
-    <row r="107" spans="2:17" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B107" s="24"/>
-      <c r="C107" s="29"/>
-      <c r="D107" s="30"/>
-      <c r="E107" s="31"/>
-      <c r="F107" s="48"/>
-      <c r="H107" s="70"/>
-      <c r="Q107" s="28"/>
-    </row>
-    <row r="108" spans="2:17" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="108" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B108" s="24"/>
       <c r="C108" s="29"/>
       <c r="D108" s="30"/>
       <c r="E108" s="31"/>
       <c r="F108" s="48"/>
-      <c r="H108" s="70"/>
-      <c r="Q108" s="28"/>
-    </row>
-    <row r="109" spans="2:17" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="109" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B109" s="24"/>
       <c r="C109" s="29"/>
       <c r="D109" s="30"/>
       <c r="E109" s="31"/>
       <c r="F109" s="48"/>
-      <c r="H109" s="70"/>
-      <c r="Q109" s="28"/>
-    </row>
-    <row r="110" spans="2:17" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B110" s="24"/>
+    </row>
+    <row r="110" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B110" s="75"/>
       <c r="C110" s="29"/>
       <c r="D110" s="30"/>
-      <c r="E110" s="32"/>
+      <c r="E110" s="31"/>
       <c r="F110" s="48"/>
-      <c r="H110" s="70"/>
-      <c r="Q110" s="28"/>
-    </row>
-    <row r="111" spans="2:17" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B111" s="27" t="s">
-        <v>20</v>
-      </c>
-      <c r="C111" s="27"/>
-      <c r="D111" s="27"/>
-      <c r="E111" s="27"/>
-      <c r="F111" s="47">
-        <f>SUM(F103:F110)</f>
-        <v>0</v>
-      </c>
-      <c r="H111" s="70"/>
-      <c r="Q111" s="28"/>
-    </row>
-    <row r="113" spans="2:17" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B113" s="79" t="s">
-        <v>40</v>
-      </c>
-      <c r="C113" s="80"/>
-      <c r="D113" s="80"/>
-      <c r="E113" s="80"/>
-      <c r="F113" s="80"/>
+    </row>
+    <row r="111" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B111" s="24"/>
+      <c r="C111" s="29"/>
+      <c r="D111" s="30"/>
+      <c r="E111" s="31"/>
+      <c r="F111" s="48"/>
+    </row>
+    <row r="112" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B112" s="24"/>
+      <c r="C112" s="29"/>
+      <c r="D112" s="30"/>
+      <c r="E112" s="31"/>
+      <c r="F112" s="48"/>
+    </row>
+    <row r="113" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B113" s="24"/>
+      <c r="C113" s="29"/>
+      <c r="D113" s="30"/>
+      <c r="E113" s="31"/>
+      <c r="F113" s="48"/>
     </row>
     <row r="114" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B114" s="81" t="s">
-        <v>9</v>
-      </c>
-      <c r="C114" s="82"/>
-      <c r="D114" s="82"/>
-      <c r="E114" s="83" t="s">
-        <v>0</v>
-      </c>
-      <c r="F114" s="83" t="s">
-        <v>10</v>
-      </c>
+      <c r="B114" s="24"/>
+      <c r="C114" s="29"/>
+      <c r="D114" s="30"/>
+      <c r="E114" s="31"/>
+      <c r="F114" s="48"/>
     </row>
     <row r="115" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B115" s="24"/>
@@ -2837,38 +2886,38 @@
       <c r="F115" s="48"/>
     </row>
     <row r="116" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B116" s="33"/>
-      <c r="C116" s="34"/>
-      <c r="D116" s="35"/>
-      <c r="E116" s="36"/>
+      <c r="B116" s="24"/>
+      <c r="C116" s="29"/>
+      <c r="D116" s="30"/>
+      <c r="E116" s="31"/>
       <c r="F116" s="48"/>
     </row>
     <row r="117" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B117" s="33"/>
+      <c r="B117" s="24"/>
       <c r="C117" s="29"/>
       <c r="D117" s="30"/>
-      <c r="E117" s="36"/>
+      <c r="E117" s="31"/>
       <c r="F117" s="48"/>
     </row>
     <row r="118" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B118" s="33"/>
+      <c r="B118" s="24"/>
       <c r="C118" s="29"/>
       <c r="D118" s="30"/>
-      <c r="E118" s="36"/>
+      <c r="E118" s="31"/>
       <c r="F118" s="48"/>
     </row>
     <row r="119" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B119" s="33"/>
+      <c r="B119" s="24"/>
       <c r="C119" s="29"/>
       <c r="D119" s="30"/>
-      <c r="E119" s="36"/>
+      <c r="E119" s="31"/>
       <c r="F119" s="48"/>
     </row>
     <row r="120" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B120" s="33"/>
+      <c r="B120" s="24"/>
       <c r="C120" s="29"/>
       <c r="D120" s="30"/>
-      <c r="E120" s="36"/>
+      <c r="E120" s="31"/>
       <c r="F120" s="48"/>
     </row>
     <row r="121" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -2878,169 +2927,613 @@
       <c r="E121" s="32"/>
       <c r="F121" s="48"/>
     </row>
-    <row r="122" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B122" s="24"/>
-      <c r="C122" s="29"/>
-      <c r="D122" s="30"/>
-      <c r="E122" s="32"/>
-      <c r="F122" s="49"/>
+    <row r="122" spans="2:17" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B122" s="74" t="s">
+        <v>20</v>
+      </c>
+      <c r="C122" s="27"/>
+      <c r="D122" s="27"/>
+      <c r="E122" s="27"/>
+      <c r="F122" s="47">
+        <f>SUM(F108:F121)</f>
+        <v>0</v>
+      </c>
+      <c r="H122" s="70"/>
+      <c r="Q122" s="28"/>
     </row>
     <row r="123" spans="2:17" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B123" s="27" t="s">
-        <v>21</v>
-      </c>
-      <c r="C123" s="27"/>
-      <c r="D123" s="27"/>
-      <c r="E123" s="27"/>
-      <c r="F123" s="47">
-        <f>SUM(F115:F122)</f>
-        <v>0</v>
-      </c>
+      <c r="F123" s="64"/>
       <c r="H123" s="70"/>
       <c r="Q123" s="28"/>
     </row>
-    <row r="125" spans="2:17" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B125" s="79" t="s">
+    <row r="124" spans="2:17" s="10" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B124" s="79" t="s">
+        <v>39</v>
+      </c>
+      <c r="C124" s="80"/>
+      <c r="D124" s="80"/>
+      <c r="E124" s="80"/>
+      <c r="F124" s="80"/>
+      <c r="H124" s="70"/>
+      <c r="Q124" s="28"/>
+    </row>
+    <row r="125" spans="2:17" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B125" s="81" t="s">
+        <v>9</v>
+      </c>
+      <c r="C125" s="82"/>
+      <c r="D125" s="82"/>
+      <c r="E125" s="83" t="s">
+        <v>0</v>
+      </c>
+      <c r="F125" s="83" t="s">
+        <v>10</v>
+      </c>
+      <c r="H125" s="70"/>
+      <c r="Q125" s="28"/>
+    </row>
+    <row r="126" spans="2:17" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B126" s="24"/>
+      <c r="C126" s="29"/>
+      <c r="D126" s="30"/>
+      <c r="E126" s="31"/>
+      <c r="F126" s="48"/>
+      <c r="H126" s="66"/>
+      <c r="Q126" s="28"/>
+    </row>
+    <row r="127" spans="2:17" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B127" s="24"/>
+      <c r="C127" s="29"/>
+      <c r="D127" s="30"/>
+      <c r="E127" s="31"/>
+      <c r="F127" s="48"/>
+      <c r="H127" s="66"/>
+      <c r="Q127" s="28"/>
+    </row>
+    <row r="128" spans="2:17" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B128" s="24"/>
+      <c r="C128" s="29"/>
+      <c r="D128" s="30"/>
+      <c r="E128" s="31"/>
+      <c r="F128" s="48"/>
+      <c r="H128" s="66"/>
+      <c r="Q128" s="28"/>
+    </row>
+    <row r="129" spans="2:17" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B129" s="24"/>
+      <c r="C129" s="29"/>
+      <c r="D129" s="30"/>
+      <c r="E129" s="31"/>
+      <c r="F129" s="48"/>
+      <c r="H129" s="66"/>
+      <c r="Q129" s="28"/>
+    </row>
+    <row r="130" spans="2:17" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B130" s="24"/>
+      <c r="C130" s="29"/>
+      <c r="D130" s="30"/>
+      <c r="E130" s="31"/>
+      <c r="F130" s="48"/>
+      <c r="H130" s="66"/>
+      <c r="Q130" s="28"/>
+    </row>
+    <row r="131" spans="2:17" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B131" s="24"/>
+      <c r="C131" s="29"/>
+      <c r="D131" s="30"/>
+      <c r="E131" s="31"/>
+      <c r="F131" s="48"/>
+      <c r="H131" s="66"/>
+      <c r="Q131" s="28"/>
+    </row>
+    <row r="132" spans="2:17" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B132" s="24"/>
+      <c r="C132" s="29"/>
+      <c r="D132" s="30"/>
+      <c r="E132" s="31"/>
+      <c r="F132" s="48"/>
+      <c r="H132" s="66"/>
+      <c r="Q132" s="28"/>
+    </row>
+    <row r="133" spans="2:17" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B133" s="24"/>
+      <c r="C133" s="29"/>
+      <c r="D133" s="30"/>
+      <c r="E133" s="31"/>
+      <c r="F133" s="48"/>
+      <c r="H133" s="66"/>
+      <c r="Q133" s="28"/>
+    </row>
+    <row r="134" spans="2:17" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B134" s="24"/>
+      <c r="C134" s="29"/>
+      <c r="D134" s="30"/>
+      <c r="E134" s="31"/>
+      <c r="F134" s="48"/>
+      <c r="H134" s="66"/>
+      <c r="Q134" s="28"/>
+    </row>
+    <row r="135" spans="2:17" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B135" s="24"/>
+      <c r="C135" s="29"/>
+      <c r="D135" s="30"/>
+      <c r="E135" s="31"/>
+      <c r="F135" s="48"/>
+      <c r="H135" s="66"/>
+      <c r="Q135" s="28"/>
+    </row>
+    <row r="136" spans="2:17" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B136" s="24"/>
+      <c r="C136" s="29"/>
+      <c r="D136" s="30"/>
+      <c r="E136" s="31"/>
+      <c r="F136" s="48"/>
+      <c r="H136" s="66"/>
+      <c r="Q136" s="28"/>
+    </row>
+    <row r="137" spans="2:17" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B137" s="24"/>
+      <c r="C137" s="29"/>
+      <c r="D137" s="30"/>
+      <c r="E137" s="31"/>
+      <c r="F137" s="48"/>
+      <c r="H137" s="66"/>
+      <c r="Q137" s="28"/>
+    </row>
+    <row r="138" spans="2:17" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B138" s="24"/>
+      <c r="C138" s="29"/>
+      <c r="D138" s="30"/>
+      <c r="E138" s="31"/>
+      <c r="F138" s="48"/>
+      <c r="H138" s="70"/>
+      <c r="Q138" s="28"/>
+    </row>
+    <row r="139" spans="2:17" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B139" s="24"/>
+      <c r="C139" s="29"/>
+      <c r="D139" s="30"/>
+      <c r="E139" s="31"/>
+      <c r="F139" s="48"/>
+      <c r="H139" s="70"/>
+      <c r="Q139" s="28"/>
+    </row>
+    <row r="140" spans="2:17" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B140" s="24"/>
+      <c r="C140" s="29"/>
+      <c r="D140" s="30"/>
+      <c r="E140" s="31"/>
+      <c r="F140" s="48"/>
+      <c r="H140" s="70"/>
+      <c r="Q140" s="28"/>
+    </row>
+    <row r="141" spans="2:17" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B141" s="24"/>
+      <c r="C141" s="29"/>
+      <c r="D141" s="30"/>
+      <c r="E141" s="31"/>
+      <c r="F141" s="48"/>
+      <c r="H141" s="70"/>
+      <c r="Q141" s="28"/>
+    </row>
+    <row r="142" spans="2:17" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B142" s="24"/>
+      <c r="C142" s="29"/>
+      <c r="D142" s="30"/>
+      <c r="E142" s="32"/>
+      <c r="F142" s="48"/>
+      <c r="H142" s="70"/>
+      <c r="Q142" s="28"/>
+    </row>
+    <row r="143" spans="2:17" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B143" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="C143" s="27"/>
+      <c r="D143" s="27"/>
+      <c r="E143" s="27"/>
+      <c r="F143" s="47">
+        <f>SUM(F126:F142)</f>
+        <v>0</v>
+      </c>
+      <c r="H143" s="70"/>
+      <c r="Q143" s="28"/>
+    </row>
+    <row r="145" spans="2:6" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B145" s="79" t="s">
+        <v>40</v>
+      </c>
+      <c r="C145" s="80"/>
+      <c r="D145" s="80"/>
+      <c r="E145" s="80"/>
+      <c r="F145" s="80"/>
+    </row>
+    <row r="146" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B146" s="81" t="s">
+        <v>9</v>
+      </c>
+      <c r="C146" s="82"/>
+      <c r="D146" s="82"/>
+      <c r="E146" s="83" t="s">
+        <v>0</v>
+      </c>
+      <c r="F146" s="83" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="147" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B147" s="24"/>
+      <c r="C147" s="29"/>
+      <c r="D147" s="30"/>
+      <c r="E147" s="31"/>
+      <c r="F147" s="48"/>
+    </row>
+    <row r="148" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B148" s="33"/>
+      <c r="C148" s="34"/>
+      <c r="D148" s="35"/>
+      <c r="E148" s="36"/>
+      <c r="F148" s="48"/>
+    </row>
+    <row r="149" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B149" s="33"/>
+      <c r="C149" s="29"/>
+      <c r="D149" s="30"/>
+      <c r="E149" s="36"/>
+      <c r="F149" s="48"/>
+    </row>
+    <row r="150" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B150" s="33"/>
+      <c r="C150" s="29"/>
+      <c r="D150" s="30"/>
+      <c r="E150" s="36"/>
+      <c r="F150" s="48"/>
+    </row>
+    <row r="151" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B151" s="33"/>
+      <c r="C151" s="29"/>
+      <c r="D151" s="30"/>
+      <c r="E151" s="36"/>
+      <c r="F151" s="48"/>
+    </row>
+    <row r="152" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B152" s="33"/>
+      <c r="C152" s="29"/>
+      <c r="D152" s="30"/>
+      <c r="E152" s="36"/>
+      <c r="F152" s="48"/>
+    </row>
+    <row r="153" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B153" s="33"/>
+      <c r="C153" s="29"/>
+      <c r="D153" s="30"/>
+      <c r="E153" s="36"/>
+      <c r="F153" s="48"/>
+    </row>
+    <row r="154" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B154" s="33"/>
+      <c r="C154" s="29"/>
+      <c r="D154" s="30"/>
+      <c r="E154" s="36"/>
+      <c r="F154" s="48"/>
+    </row>
+    <row r="155" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B155" s="33"/>
+      <c r="C155" s="29"/>
+      <c r="D155" s="30"/>
+      <c r="E155" s="36"/>
+      <c r="F155" s="48"/>
+    </row>
+    <row r="156" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B156" s="33"/>
+      <c r="C156" s="29"/>
+      <c r="D156" s="30"/>
+      <c r="E156" s="36"/>
+      <c r="F156" s="48"/>
+    </row>
+    <row r="157" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B157" s="33"/>
+      <c r="C157" s="29"/>
+      <c r="D157" s="30"/>
+      <c r="E157" s="36"/>
+      <c r="F157" s="48"/>
+    </row>
+    <row r="158" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B158" s="33"/>
+      <c r="C158" s="29"/>
+      <c r="D158" s="30"/>
+      <c r="E158" s="36"/>
+      <c r="F158" s="48"/>
+    </row>
+    <row r="159" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B159" s="33"/>
+      <c r="C159" s="29"/>
+      <c r="D159" s="30"/>
+      <c r="E159" s="36"/>
+      <c r="F159" s="48"/>
+    </row>
+    <row r="160" spans="2:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B160" s="33"/>
+      <c r="C160" s="29"/>
+      <c r="D160" s="30"/>
+      <c r="E160" s="36"/>
+      <c r="F160" s="48"/>
+    </row>
+    <row r="161" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B161" s="33"/>
+      <c r="C161" s="29"/>
+      <c r="D161" s="30"/>
+      <c r="E161" s="36"/>
+      <c r="F161" s="48"/>
+    </row>
+    <row r="162" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B162" s="24"/>
+      <c r="C162" s="29"/>
+      <c r="D162" s="30"/>
+      <c r="E162" s="32"/>
+      <c r="F162" s="48"/>
+    </row>
+    <row r="163" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B163" s="24"/>
+      <c r="C163" s="29"/>
+      <c r="D163" s="30"/>
+      <c r="E163" s="32"/>
+      <c r="F163" s="49"/>
+    </row>
+    <row r="164" spans="2:17" s="10" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B164" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="C164" s="27"/>
+      <c r="D164" s="27"/>
+      <c r="E164" s="27"/>
+      <c r="F164" s="47">
+        <f>SUM(F147:F163)</f>
+        <v>0</v>
+      </c>
+      <c r="H164" s="70"/>
+      <c r="Q164" s="28"/>
+    </row>
+    <row r="166" spans="2:17" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B166" s="79" t="s">
         <v>41</v>
       </c>
-      <c r="C125" s="80"/>
-      <c r="D125" s="80"/>
-      <c r="E125" s="80"/>
-      <c r="F125" s="80"/>
-    </row>
-    <row r="126" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B126" s="81" t="s">
+      <c r="C166" s="80"/>
+      <c r="D166" s="80"/>
+      <c r="E166" s="80"/>
+      <c r="F166" s="80"/>
+    </row>
+    <row r="167" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B167" s="81" t="s">
         <v>22</v>
       </c>
-      <c r="C126" s="82"/>
-      <c r="D126" s="82"/>
-      <c r="E126" s="83" t="s">
-        <v>0</v>
-      </c>
-      <c r="F126" s="83" t="s">
+      <c r="C167" s="82"/>
+      <c r="D167" s="82"/>
+      <c r="E167" s="83" t="s">
+        <v>0</v>
+      </c>
+      <c r="F167" s="83" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="127" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B127" s="33"/>
-      <c r="C127" s="34"/>
-      <c r="D127" s="35"/>
-      <c r="E127" s="31"/>
-      <c r="F127" s="50"/>
-    </row>
-    <row r="128" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B128" s="33"/>
-      <c r="C128" s="34"/>
-      <c r="D128" s="35"/>
-      <c r="E128" s="36"/>
-      <c r="F128" s="37"/>
-    </row>
-    <row r="129" spans="1:7" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B129" s="24"/>
-      <c r="C129" s="34"/>
-      <c r="D129" s="35"/>
-      <c r="E129" s="36"/>
-      <c r="F129" s="37"/>
-    </row>
-    <row r="130" spans="1:7" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B130" s="24"/>
-      <c r="C130" s="34"/>
-      <c r="D130" s="35"/>
-      <c r="E130" s="36"/>
-      <c r="F130" s="37"/>
-    </row>
-    <row r="131" spans="1:7" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B131" s="33"/>
-      <c r="C131" s="34"/>
-      <c r="D131" s="35"/>
-      <c r="E131" s="36"/>
-      <c r="F131" s="37"/>
-    </row>
-    <row r="132" spans="1:7" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B132" s="33"/>
-      <c r="C132" s="34"/>
-      <c r="D132" s="35"/>
-      <c r="E132" s="36"/>
-      <c r="F132" s="37"/>
-    </row>
-    <row r="133" spans="1:7" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B133" s="33"/>
-      <c r="C133" s="34"/>
-      <c r="D133" s="35"/>
-      <c r="E133" s="36"/>
-      <c r="F133" s="37"/>
-    </row>
-    <row r="134" spans="1:7" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B134" s="33"/>
-      <c r="C134" s="34"/>
-      <c r="D134" s="35"/>
-      <c r="E134" s="36"/>
-      <c r="F134" s="37"/>
-    </row>
-    <row r="135" spans="1:7" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B135" s="33"/>
-      <c r="C135" s="34"/>
-      <c r="D135" s="35"/>
-      <c r="E135" s="36"/>
-      <c r="F135" s="37"/>
-    </row>
-    <row r="136" spans="1:7" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B136" s="33"/>
-      <c r="C136" s="34"/>
-      <c r="D136" s="35"/>
-      <c r="E136" s="36"/>
-      <c r="F136" s="37"/>
-    </row>
-    <row r="137" spans="1:7" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B137" s="38" t="s">
+    <row r="168" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B168" s="33"/>
+      <c r="C168" s="34"/>
+      <c r="D168" s="35"/>
+      <c r="E168" s="31"/>
+      <c r="F168" s="50"/>
+    </row>
+    <row r="169" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B169" s="33"/>
+      <c r="C169" s="34"/>
+      <c r="D169" s="35"/>
+      <c r="E169" s="36"/>
+      <c r="F169" s="37"/>
+    </row>
+    <row r="170" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B170" s="24"/>
+      <c r="C170" s="34"/>
+      <c r="D170" s="35"/>
+      <c r="E170" s="36"/>
+      <c r="F170" s="37"/>
+      <c r="H170" s="4"/>
+      <c r="Q170" s="4"/>
+    </row>
+    <row r="171" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B171" s="24"/>
+      <c r="C171" s="34"/>
+      <c r="D171" s="35"/>
+      <c r="E171" s="36"/>
+      <c r="F171" s="37"/>
+      <c r="H171" s="4"/>
+      <c r="Q171" s="4"/>
+    </row>
+    <row r="172" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B172" s="33"/>
+      <c r="C172" s="34"/>
+      <c r="D172" s="35"/>
+      <c r="E172" s="36"/>
+      <c r="F172" s="37"/>
+      <c r="H172" s="4"/>
+      <c r="Q172" s="4"/>
+    </row>
+    <row r="173" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B173" s="33"/>
+      <c r="C173" s="34"/>
+      <c r="D173" s="35"/>
+      <c r="E173" s="36"/>
+      <c r="F173" s="37"/>
+      <c r="H173" s="4"/>
+      <c r="Q173" s="4"/>
+    </row>
+    <row r="174" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B174" s="33"/>
+      <c r="C174" s="34"/>
+      <c r="D174" s="35"/>
+      <c r="E174" s="36"/>
+      <c r="F174" s="37"/>
+      <c r="H174" s="4"/>
+      <c r="Q174" s="4"/>
+    </row>
+    <row r="175" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B175" s="33"/>
+      <c r="C175" s="34"/>
+      <c r="D175" s="35"/>
+      <c r="E175" s="36"/>
+      <c r="F175" s="37"/>
+      <c r="H175" s="4"/>
+      <c r="Q175" s="4"/>
+    </row>
+    <row r="176" spans="2:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B176" s="33"/>
+      <c r="C176" s="34"/>
+      <c r="D176" s="35"/>
+      <c r="E176" s="36"/>
+      <c r="F176" s="37"/>
+      <c r="H176" s="4"/>
+      <c r="Q176" s="4"/>
+    </row>
+    <row r="177" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B177" s="33"/>
+      <c r="C177" s="34"/>
+      <c r="D177" s="35"/>
+      <c r="E177" s="36"/>
+      <c r="F177" s="37"/>
+      <c r="H177" s="4"/>
+      <c r="Q177" s="4"/>
+    </row>
+    <row r="178" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B178" s="33"/>
+      <c r="C178" s="34"/>
+      <c r="D178" s="35"/>
+      <c r="E178" s="36"/>
+      <c r="F178" s="37"/>
+      <c r="H178" s="4"/>
+      <c r="Q178" s="4"/>
+    </row>
+    <row r="179" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B179" s="33"/>
+      <c r="C179" s="34"/>
+      <c r="D179" s="35"/>
+      <c r="E179" s="36"/>
+      <c r="F179" s="37"/>
+      <c r="H179" s="4"/>
+      <c r="Q179" s="4"/>
+    </row>
+    <row r="180" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B180" s="33"/>
+      <c r="C180" s="34"/>
+      <c r="D180" s="35"/>
+      <c r="E180" s="36"/>
+      <c r="F180" s="37"/>
+      <c r="H180" s="4"/>
+      <c r="Q180" s="4"/>
+    </row>
+    <row r="181" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B181" s="33"/>
+      <c r="C181" s="34"/>
+      <c r="D181" s="35"/>
+      <c r="E181" s="36"/>
+      <c r="F181" s="37"/>
+      <c r="H181" s="4"/>
+      <c r="Q181" s="4"/>
+    </row>
+    <row r="182" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B182" s="33"/>
+      <c r="C182" s="34"/>
+      <c r="D182" s="35"/>
+      <c r="E182" s="36"/>
+      <c r="F182" s="37"/>
+      <c r="H182" s="4"/>
+      <c r="Q182" s="4"/>
+    </row>
+    <row r="183" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B183" s="33"/>
+      <c r="C183" s="34"/>
+      <c r="D183" s="35"/>
+      <c r="E183" s="36"/>
+      <c r="F183" s="37"/>
+      <c r="H183" s="4"/>
+      <c r="Q183" s="4"/>
+    </row>
+    <row r="184" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B184" s="33"/>
+      <c r="C184" s="34"/>
+      <c r="D184" s="35"/>
+      <c r="E184" s="36"/>
+      <c r="F184" s="37"/>
+      <c r="H184" s="4"/>
+      <c r="Q184" s="4"/>
+    </row>
+    <row r="185" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B185" s="33"/>
+      <c r="C185" s="34"/>
+      <c r="D185" s="35"/>
+      <c r="E185" s="36"/>
+      <c r="F185" s="37"/>
+      <c r="H185" s="4"/>
+      <c r="Q185" s="4"/>
+    </row>
+    <row r="186" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B186" s="38" t="s">
         <v>23</v>
       </c>
-      <c r="C137" s="38"/>
-      <c r="D137" s="38"/>
-      <c r="E137" s="38"/>
-      <c r="F137" s="51">
-        <f>SUM(F127:F136)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="138" spans="1:7" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A138" s="4" t="s">
+      <c r="C186" s="38"/>
+      <c r="D186" s="38"/>
+      <c r="E186" s="38"/>
+      <c r="F186" s="51">
+        <f>SUM(F168:F185)</f>
+        <v>0</v>
+      </c>
+      <c r="H186" s="4"/>
+      <c r="Q186" s="4"/>
+    </row>
+    <row r="187" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A187" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="B138" s="39"/>
-      <c r="C138" s="39"/>
-      <c r="D138" s="39"/>
-      <c r="E138" s="39"/>
-      <c r="F138" s="40"/>
-      <c r="G138" s="4" t="s">
+      <c r="B187" s="39"/>
+      <c r="C187" s="39"/>
+      <c r="D187" s="39"/>
+      <c r="E187" s="39"/>
+      <c r="F187" s="40"/>
+      <c r="G187" s="4" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="139" spans="1:7" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B139" s="1"/>
-      <c r="C139" s="1"/>
-      <c r="D139" s="1"/>
-      <c r="E139" s="1"/>
-      <c r="F139" s="41"/>
-    </row>
-    <row r="140" spans="1:7" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B140" s="42"/>
-      <c r="C140" s="1"/>
-      <c r="D140" s="1"/>
-      <c r="E140" s="1"/>
-      <c r="F140" s="43"/>
-    </row>
-    <row r="141" spans="1:7" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B141" s="42"/>
-      <c r="F141" s="46"/>
+      <c r="H187" s="4"/>
+      <c r="Q187" s="4"/>
+    </row>
+    <row r="188" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B188" s="1"/>
+      <c r="C188" s="1"/>
+      <c r="D188" s="1"/>
+      <c r="E188" s="1"/>
+      <c r="F188" s="41"/>
+      <c r="H188" s="4"/>
+      <c r="Q188" s="4"/>
+    </row>
+    <row r="189" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B189" s="42"/>
+      <c r="C189" s="1"/>
+      <c r="D189" s="1"/>
+      <c r="E189" s="1"/>
+      <c r="F189" s="43"/>
+      <c r="H189" s="4"/>
+      <c r="Q189" s="4"/>
+    </row>
+    <row r="190" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B190" s="42"/>
+      <c r="F190" s="46"/>
+      <c r="H190" s="4"/>
+      <c r="Q190" s="4"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="F81:F87">
+  <conditionalFormatting sqref="F90:F104">
     <cfRule type="cellIs" dxfId="1" priority="2" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F141">
+  <conditionalFormatting sqref="F190">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="notBetween">
       <formula>0.1</formula>
       <formula>-0.1</formula>

</xml_diff>